<commit_message>
update WCR dashboard data 2026-07-01 10:51
</commit_message>
<xml_diff>
--- a/docs/reports/WCR_Kavach_Unified_KPI_Jun1-Jun7.xlsx
+++ b/docs/reports/WCR_Kavach_Unified_KPI_Jun1-Jun7.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="#,##0.0"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.00000"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -184,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -206,13 +206,13 @@
     <xf numFmtId="3" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -228,7 +228,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -243,7 +243,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -258,7 +258,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -308,6 +308,24 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -856,19 +874,19 @@
         <f>'Daily Breakdown'!J253</f>
         <v/>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="46">
         <f>IFERROR(G5/D5,0)</f>
         <v/>
       </c>
-      <c r="K5" s="10">
+      <c r="K5" s="47">
         <f>IFERROR(G5/E5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="48">
         <f>IFERROR(G5/E5*100,0)</f>
         <v/>
       </c>
-      <c r="M5" s="10">
+      <c r="M5" s="47">
         <f>IFERROR(G5/(D5*E5/1000),0)</f>
         <v/>
       </c>
@@ -876,24 +894,24 @@
         <f>'Daily Breakdown'!K253</f>
         <v/>
       </c>
-      <c r="O5" s="9">
+      <c r="O5" s="46">
         <f>IFERROR(N5/D5,0)</f>
         <v/>
       </c>
-      <c r="P5" s="10">
+      <c r="P5" s="47">
         <f>IFERROR(N5/E5,0)</f>
         <v/>
       </c>
-      <c r="Q5" s="10">
+      <c r="Q5" s="47">
         <f>IFERROR(N5/(D5*E5/100),0)</f>
         <v/>
       </c>
-      <c r="R5" s="11">
+      <c r="R5" s="48">
         <f>IFERROR(N5/E5*100,0)</f>
         <v/>
       </c>
       <c r="S5" s="8" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="T5" s="12">
         <f>ROUND(F5*(1-M5)*(1-Q5),2)</f>
@@ -938,7 +956,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -1010,7 +1027,7 @@
       <c r="C4" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="17" t="n">
+      <c r="D4" s="49" t="n">
         <v>543.9</v>
       </c>
       <c r="E4" s="18" t="n">
@@ -1050,7 +1067,7 @@
       <c r="C5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="49" t="n">
         <v>541.66</v>
       </c>
       <c r="E5" s="18" t="n">
@@ -1090,7 +1107,7 @@
       <c r="C6" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="49" t="n">
         <v>543.88</v>
       </c>
       <c r="E6" s="18" t="n">
@@ -1130,7 +1147,7 @@
       <c r="C7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="49" t="n">
         <v>543.61</v>
       </c>
       <c r="E7" s="18" t="n">
@@ -1170,7 +1187,7 @@
       <c r="C8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="49" t="n">
         <v>541.62</v>
       </c>
       <c r="E8" s="18" t="n">
@@ -1210,7 +1227,7 @@
       <c r="C9" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="49" t="n">
         <v>251.78</v>
       </c>
       <c r="E9" s="18" t="n">
@@ -1250,7 +1267,7 @@
       <c r="C10" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="49" t="n">
         <v>251.84</v>
       </c>
       <c r="E10" s="18" t="n">
@@ -1290,7 +1307,7 @@
       <c r="C11" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="D11" s="49" t="n">
         <v>322.32</v>
       </c>
       <c r="E11" s="18" t="n">
@@ -1330,7 +1347,7 @@
       <c r="C12" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="49" t="n">
         <v>321.48</v>
       </c>
       <c r="E12" s="18" t="n">
@@ -1370,7 +1387,7 @@
       <c r="C13" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="49" t="n">
         <v>388.48</v>
       </c>
       <c r="E13" s="18" t="n">
@@ -1410,7 +1427,7 @@
       <c r="C14" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="49" t="n">
         <v>454.04</v>
       </c>
       <c r="E14" s="18" t="n">
@@ -1450,7 +1467,7 @@
       <c r="C15" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="49" t="n">
         <v>470.6</v>
       </c>
       <c r="E15" s="18" t="n">
@@ -1490,7 +1507,7 @@
       <c r="C16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="49" t="n">
         <v>346.04</v>
       </c>
       <c r="E16" s="18" t="n">
@@ -1530,7 +1547,7 @@
       <c r="C17" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="17" t="n">
+      <c r="D17" s="49" t="n">
         <v>330.73</v>
       </c>
       <c r="E17" s="18" t="n">
@@ -1570,7 +1587,7 @@
       <c r="C18" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="49" t="n">
         <v>108.66</v>
       </c>
       <c r="E18" s="18" t="n">
@@ -1610,7 +1627,7 @@
       <c r="C19" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="17" t="n">
+      <c r="D19" s="49" t="n">
         <v>235.98</v>
       </c>
       <c r="E19" s="18" t="n">
@@ -1650,7 +1667,7 @@
       <c r="C20" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="49" t="n">
         <v>319.21</v>
       </c>
       <c r="E20" s="18" t="n">
@@ -1690,7 +1707,7 @@
       <c r="C21" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D21" s="17" t="n">
+      <c r="D21" s="49" t="n">
         <v>319.25</v>
       </c>
       <c r="E21" s="18" t="n">
@@ -1730,7 +1747,7 @@
       <c r="C22" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="49" t="n">
         <v>108.53</v>
       </c>
       <c r="E22" s="18" t="n">
@@ -1770,7 +1787,7 @@
       <c r="C23" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="17" t="n">
+      <c r="D23" s="49" t="n">
         <v>319.23</v>
       </c>
       <c r="E23" s="18" t="n">
@@ -1810,7 +1827,7 @@
       <c r="C24" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="49" t="n">
         <v>251.19</v>
       </c>
       <c r="E24" s="18" t="n">
@@ -1850,7 +1867,7 @@
       <c r="C25" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="17" t="n">
+      <c r="D25" s="49" t="n">
         <v>150.97</v>
       </c>
       <c r="E25" s="18" t="n">
@@ -1890,7 +1907,7 @@
       <c r="C26" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="17" t="n">
+      <c r="D26" s="49" t="n">
         <v>217.38</v>
       </c>
       <c r="E26" s="18" t="n">
@@ -1930,7 +1947,7 @@
       <c r="C27" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="49" t="n">
         <v>307.65</v>
       </c>
       <c r="E27" s="18" t="n">
@@ -1970,7 +1987,7 @@
       <c r="C28" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="49" t="n">
         <v>87.36</v>
       </c>
       <c r="E28" s="18" t="n">
@@ -2010,7 +2027,7 @@
       <c r="C29" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D29" s="49" t="n">
         <v>26.91</v>
       </c>
       <c r="E29" s="18" t="n">
@@ -2050,7 +2067,7 @@
       <c r="C30" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="49" t="n">
         <v>53.57</v>
       </c>
       <c r="E30" s="18" t="n">
@@ -2090,7 +2107,7 @@
       <c r="C31" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="17" t="n">
+      <c r="D31" s="49" t="n">
         <v>46.88</v>
       </c>
       <c r="E31" s="18" t="n">
@@ -2130,7 +2147,7 @@
       <c r="C32" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D32" s="17" t="n">
+      <c r="D32" s="49" t="n">
         <v>222.32</v>
       </c>
       <c r="E32" s="18" t="n">
@@ -2170,7 +2187,7 @@
       <c r="C33" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D33" s="17" t="n">
+      <c r="D33" s="49" t="n">
         <v>41.17</v>
       </c>
       <c r="E33" s="18" t="n">
@@ -2210,7 +2227,7 @@
       <c r="C34" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D34" s="17" t="n">
+      <c r="D34" s="49" t="n">
         <v>13.96</v>
       </c>
       <c r="E34" s="18" t="n">
@@ -2250,7 +2267,7 @@
       <c r="C35" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D35" s="17" t="n">
+      <c r="D35" s="49" t="n">
         <v>2.88</v>
       </c>
       <c r="E35" s="18" t="n">
@@ -2290,7 +2307,7 @@
       <c r="C36" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D36" s="17" t="n">
+      <c r="D36" s="49" t="n">
         <v>61.41</v>
       </c>
       <c r="E36" s="18" t="n">
@@ -2330,7 +2347,7 @@
       <c r="C37" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D37" s="17" t="n">
+      <c r="D37" s="49" t="n">
         <v>112.1</v>
       </c>
       <c r="E37" s="18" t="n">
@@ -2370,7 +2387,7 @@
       <c r="C38" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="17" t="n">
+      <c r="D38" s="49" t="n">
         <v>107.54</v>
       </c>
       <c r="E38" s="18" t="n">
@@ -2411,7 +2428,7 @@
         <f>SUM(C4:C38)</f>
         <v/>
       </c>
-      <c r="D39" s="22">
+      <c r="D39" s="50">
         <f>SUM(D4:D38)</f>
         <v/>
       </c>
@@ -2458,7 +2475,7 @@
       <c r="C40" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D40" s="17" t="n">
+      <c r="D40" s="49" t="n">
         <v>543.66</v>
       </c>
       <c r="E40" s="18" t="n">
@@ -2498,7 +2515,7 @@
       <c r="C41" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="17" t="n">
+      <c r="D41" s="49" t="n">
         <v>543.89</v>
       </c>
       <c r="E41" s="18" t="n">
@@ -2538,7 +2555,7 @@
       <c r="C42" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D42" s="17" t="n">
+      <c r="D42" s="49" t="n">
         <v>543.85</v>
       </c>
       <c r="E42" s="18" t="n">
@@ -2578,7 +2595,7 @@
       <c r="C43" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D43" s="17" t="n">
+      <c r="D43" s="49" t="n">
         <v>251.89</v>
       </c>
       <c r="E43" s="18" t="n">
@@ -2618,7 +2635,7 @@
       <c r="C44" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D44" s="17" t="n">
+      <c r="D44" s="49" t="n">
         <v>485.71</v>
       </c>
       <c r="E44" s="18" t="n">
@@ -2658,7 +2675,7 @@
       <c r="C45" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D45" s="17" t="n">
+      <c r="D45" s="49" t="n">
         <v>392.9</v>
       </c>
       <c r="E45" s="18" t="n">
@@ -2698,7 +2715,7 @@
       <c r="C46" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D46" s="17" t="n">
+      <c r="D46" s="49" t="n">
         <v>243.1</v>
       </c>
       <c r="E46" s="18" t="n">
@@ -2738,7 +2755,7 @@
       <c r="C47" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D47" s="17" t="n">
+      <c r="D47" s="49" t="n">
         <v>474.05</v>
       </c>
       <c r="E47" s="18" t="n">
@@ -2778,7 +2795,7 @@
       <c r="C48" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D48" s="17" t="n">
+      <c r="D48" s="49" t="n">
         <v>525.37</v>
       </c>
       <c r="E48" s="18" t="n">
@@ -2818,7 +2835,7 @@
       <c r="C49" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D49" s="17" t="n">
+      <c r="D49" s="49" t="n">
         <v>330.96</v>
       </c>
       <c r="E49" s="18" t="n">
@@ -2858,7 +2875,7 @@
       <c r="C50" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D50" s="17" t="n">
+      <c r="D50" s="49" t="n">
         <v>330.67</v>
       </c>
       <c r="E50" s="18" t="n">
@@ -2898,7 +2915,7 @@
       <c r="C51" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D51" s="17" t="n">
+      <c r="D51" s="49" t="n">
         <v>322.56</v>
       </c>
       <c r="E51" s="18" t="n">
@@ -2938,7 +2955,7 @@
       <c r="C52" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D52" s="17" t="n">
+      <c r="D52" s="49" t="n">
         <v>321.71</v>
       </c>
       <c r="E52" s="18" t="n">
@@ -2978,7 +2995,7 @@
       <c r="C53" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D53" s="17" t="n">
+      <c r="D53" s="49" t="n">
         <v>329.1</v>
       </c>
       <c r="E53" s="18" t="n">
@@ -3018,7 +3035,7 @@
       <c r="C54" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D54" s="17" t="n">
+      <c r="D54" s="49" t="n">
         <v>329.82</v>
       </c>
       <c r="E54" s="18" t="n">
@@ -3058,7 +3075,7 @@
       <c r="C55" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D55" s="17" t="n">
+      <c r="D55" s="49" t="n">
         <v>318.81</v>
       </c>
       <c r="E55" s="18" t="n">
@@ -3098,7 +3115,7 @@
       <c r="C56" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D56" s="17" t="n">
+      <c r="D56" s="49" t="n">
         <v>108.55</v>
       </c>
       <c r="E56" s="18" t="n">
@@ -3138,7 +3155,7 @@
       <c r="C57" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D57" s="17" t="n">
+      <c r="D57" s="49" t="n">
         <v>256.68</v>
       </c>
       <c r="E57" s="18" t="n">
@@ -3178,7 +3195,7 @@
       <c r="C58" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D58" s="17" t="n">
+      <c r="D58" s="49" t="n">
         <v>305.68</v>
       </c>
       <c r="E58" s="18" t="n">
@@ -3218,7 +3235,7 @@
       <c r="C59" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D59" s="17" t="n">
+      <c r="D59" s="49" t="n">
         <v>104.57</v>
       </c>
       <c r="E59" s="18" t="n">
@@ -3258,7 +3275,7 @@
       <c r="C60" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D60" s="17" t="n">
+      <c r="D60" s="49" t="n">
         <v>36.96</v>
       </c>
       <c r="E60" s="18" t="n">
@@ -3298,7 +3315,7 @@
       <c r="C61" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D61" s="17" t="n">
+      <c r="D61" s="49" t="n">
         <v>39.62</v>
       </c>
       <c r="E61" s="18" t="n">
@@ -3338,7 +3355,7 @@
       <c r="C62" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D62" s="17" t="n">
+      <c r="D62" s="49" t="n">
         <v>25.98</v>
       </c>
       <c r="E62" s="18" t="n">
@@ -3378,7 +3395,7 @@
       <c r="C63" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D63" s="17" t="n">
+      <c r="D63" s="49" t="n">
         <v>32.73</v>
       </c>
       <c r="E63" s="18" t="n">
@@ -3418,7 +3435,7 @@
       <c r="C64" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D64" s="17" t="n">
+      <c r="D64" s="49" t="n">
         <v>20.71</v>
       </c>
       <c r="E64" s="18" t="n">
@@ -3458,7 +3475,7 @@
       <c r="C65" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D65" s="17" t="n">
+      <c r="D65" s="49" t="n">
         <v>3.78</v>
       </c>
       <c r="E65" s="18" t="n">
@@ -3498,7 +3515,7 @@
       <c r="C66" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D66" s="17" t="n">
+      <c r="D66" s="49" t="n">
         <v>69.22</v>
       </c>
       <c r="E66" s="18" t="n">
@@ -3538,7 +3555,7 @@
       <c r="C67" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D67" s="17" t="n">
+      <c r="D67" s="49" t="n">
         <v>108.56</v>
       </c>
       <c r="E67" s="18" t="n">
@@ -3578,7 +3595,7 @@
       <c r="C68" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D68" s="17" t="n">
+      <c r="D68" s="49" t="n">
         <v>39.64</v>
       </c>
       <c r="E68" s="18" t="n">
@@ -3619,7 +3636,7 @@
         <f>SUM(C40:C68)</f>
         <v/>
       </c>
-      <c r="D69" s="22">
+      <c r="D69" s="50">
         <f>SUM(D40:D68)</f>
         <v/>
       </c>
@@ -3666,7 +3683,7 @@
       <c r="C70" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D70" s="17" t="n">
+      <c r="D70" s="49" t="n">
         <v>543.86</v>
       </c>
       <c r="E70" s="18" t="n">
@@ -3706,7 +3723,7 @@
       <c r="C71" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D71" s="17" t="n">
+      <c r="D71" s="49" t="n">
         <v>541.65</v>
       </c>
       <c r="E71" s="18" t="n">
@@ -3746,7 +3763,7 @@
       <c r="C72" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D72" s="17" t="n">
+      <c r="D72" s="49" t="n">
         <v>541.65</v>
       </c>
       <c r="E72" s="18" t="n">
@@ -3786,7 +3803,7 @@
       <c r="C73" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D73" s="17" t="n">
+      <c r="D73" s="49" t="n">
         <v>543.88</v>
       </c>
       <c r="E73" s="18" t="n">
@@ -3826,7 +3843,7 @@
       <c r="C74" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D74" s="17" t="n">
+      <c r="D74" s="49" t="n">
         <v>543.65</v>
       </c>
       <c r="E74" s="18" t="n">
@@ -3866,7 +3883,7 @@
       <c r="C75" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D75" s="17" t="n">
+      <c r="D75" s="49" t="n">
         <v>543.8200000000001</v>
       </c>
       <c r="E75" s="18" t="n">
@@ -3906,7 +3923,7 @@
       <c r="C76" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D76" s="17" t="n">
+      <c r="D76" s="49" t="n">
         <v>251.85</v>
       </c>
       <c r="E76" s="18" t="n">
@@ -3946,7 +3963,7 @@
       <c r="C77" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D77" s="17" t="n">
+      <c r="D77" s="49" t="n">
         <v>251.76</v>
       </c>
       <c r="E77" s="18" t="n">
@@ -3986,7 +4003,7 @@
       <c r="C78" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D78" s="17" t="n">
+      <c r="D78" s="49" t="n">
         <v>321.5</v>
       </c>
       <c r="E78" s="18" t="n">
@@ -4026,7 +4043,7 @@
       <c r="C79" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D79" s="17" t="n">
+      <c r="D79" s="49" t="n">
         <v>470.58</v>
       </c>
       <c r="E79" s="18" t="n">
@@ -4066,7 +4083,7 @@
       <c r="C80" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D80" s="17" t="n">
+      <c r="D80" s="49" t="n">
         <v>537.59</v>
       </c>
       <c r="E80" s="18" t="n">
@@ -4106,7 +4123,7 @@
       <c r="C81" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D81" s="17" t="n">
+      <c r="D81" s="49" t="n">
         <v>502.1</v>
       </c>
       <c r="E81" s="18" t="n">
@@ -4146,7 +4163,7 @@
       <c r="C82" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D82" s="17" t="n">
+      <c r="D82" s="49" t="n">
         <v>319.23</v>
       </c>
       <c r="E82" s="18" t="n">
@@ -4186,7 +4203,7 @@
       <c r="C83" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D83" s="17" t="n">
+      <c r="D83" s="49" t="n">
         <v>354.81</v>
       </c>
       <c r="E83" s="18" t="n">
@@ -4226,7 +4243,7 @@
       <c r="C84" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D84" s="17" t="n">
+      <c r="D84" s="49" t="n">
         <v>392.7</v>
       </c>
       <c r="E84" s="18" t="n">
@@ -4266,7 +4283,7 @@
       <c r="C85" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D85" s="17" t="n">
+      <c r="D85" s="49" t="n">
         <v>330.33</v>
       </c>
       <c r="E85" s="18" t="n">
@@ -4306,7 +4323,7 @@
       <c r="C86" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D86" s="17" t="n">
+      <c r="D86" s="49" t="n">
         <v>319.23</v>
       </c>
       <c r="E86" s="18" t="n">
@@ -4346,7 +4363,7 @@
       <c r="C87" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D87" s="17" t="n">
+      <c r="D87" s="49" t="n">
         <v>321.73</v>
       </c>
       <c r="E87" s="18" t="n">
@@ -4386,7 +4403,7 @@
       <c r="C88" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D88" s="17" t="n">
+      <c r="D88" s="49" t="n">
         <v>212.88</v>
       </c>
       <c r="E88" s="18" t="n">
@@ -4426,7 +4443,7 @@
       <c r="C89" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D89" s="17" t="n">
+      <c r="D89" s="49" t="n">
         <v>108.54</v>
       </c>
       <c r="E89" s="18" t="n">
@@ -4466,7 +4483,7 @@
       <c r="C90" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D90" s="17" t="n">
+      <c r="D90" s="49" t="n">
         <v>221.52</v>
       </c>
       <c r="E90" s="18" t="n">
@@ -4506,7 +4523,7 @@
       <c r="C91" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D91" s="17" t="n">
+      <c r="D91" s="49" t="n">
         <v>188.92</v>
       </c>
       <c r="E91" s="18" t="n">
@@ -4546,7 +4563,7 @@
       <c r="C92" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D92" s="17" t="n">
+      <c r="D92" s="49" t="n">
         <v>107.53</v>
       </c>
       <c r="E92" s="18" t="n">
@@ -4586,7 +4603,7 @@
       <c r="C93" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D93" s="17" t="n">
+      <c r="D93" s="49" t="n">
         <v>295.06</v>
       </c>
       <c r="E93" s="18" t="n">
@@ -4626,7 +4643,7 @@
       <c r="C94" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D94" s="17" t="n">
+      <c r="D94" s="49" t="n">
         <v>102.98</v>
       </c>
       <c r="E94" s="18" t="n">
@@ -4666,7 +4683,7 @@
       <c r="C95" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D95" s="17" t="n">
+      <c r="D95" s="49" t="n">
         <v>0.85</v>
       </c>
       <c r="E95" s="18" t="n">
@@ -4706,7 +4723,7 @@
       <c r="C96" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D96" s="17" t="n">
+      <c r="D96" s="49" t="n">
         <v>36.9</v>
       </c>
       <c r="E96" s="18" t="n">
@@ -4746,7 +4763,7 @@
       <c r="C97" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D97" s="17" t="n">
+      <c r="D97" s="49" t="n">
         <v>15.48</v>
       </c>
       <c r="E97" s="18" t="n">
@@ -4786,7 +4803,7 @@
       <c r="C98" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D98" s="17" t="n">
+      <c r="D98" s="49" t="n">
         <v>3.09</v>
       </c>
       <c r="E98" s="18" t="n">
@@ -4826,7 +4843,7 @@
       <c r="C99" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D99" s="17" t="n">
+      <c r="D99" s="49" t="n">
         <v>19.7</v>
       </c>
       <c r="E99" s="18" t="n">
@@ -4866,7 +4883,7 @@
       <c r="C100" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D100" s="17" t="n">
+      <c r="D100" s="49" t="n">
         <v>105.67</v>
       </c>
       <c r="E100" s="18" t="n">
@@ -4907,7 +4924,7 @@
         <f>SUM(C70:C100)</f>
         <v/>
       </c>
-      <c r="D101" s="22">
+      <c r="D101" s="50">
         <f>SUM(D70:D100)</f>
         <v/>
       </c>
@@ -4954,7 +4971,7 @@
       <c r="C102" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D102" s="17" t="n">
+      <c r="D102" s="49" t="n">
         <v>543.83</v>
       </c>
       <c r="E102" s="18" t="n">
@@ -4994,7 +5011,7 @@
       <c r="C103" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D103" s="17" t="n">
+      <c r="D103" s="49" t="n">
         <v>543.88</v>
       </c>
       <c r="E103" s="18" t="n">
@@ -5034,7 +5051,7 @@
       <c r="C104" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D104" s="17" t="n">
+      <c r="D104" s="49" t="n">
         <v>543.9</v>
       </c>
       <c r="E104" s="18" t="n">
@@ -5074,7 +5091,7 @@
       <c r="C105" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D105" s="17" t="n">
+      <c r="D105" s="49" t="n">
         <v>541.64</v>
       </c>
       <c r="E105" s="18" t="n">
@@ -5114,7 +5131,7 @@
       <c r="C106" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D106" s="17" t="n">
+      <c r="D106" s="49" t="n">
         <v>540.89</v>
       </c>
       <c r="E106" s="18" t="n">
@@ -5154,7 +5171,7 @@
       <c r="C107" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D107" s="17" t="n">
+      <c r="D107" s="49" t="n">
         <v>251.86</v>
       </c>
       <c r="E107" s="18" t="n">
@@ -5194,7 +5211,7 @@
       <c r="C108" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D108" s="17" t="n">
+      <c r="D108" s="49" t="n">
         <v>322.61</v>
       </c>
       <c r="E108" s="18" t="n">
@@ -5234,7 +5251,7 @@
       <c r="C109" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D109" s="17" t="n">
+      <c r="D109" s="49" t="n">
         <v>527.42</v>
       </c>
       <c r="E109" s="18" t="n">
@@ -5274,7 +5291,7 @@
       <c r="C110" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D110" s="17" t="n">
+      <c r="D110" s="49" t="n">
         <v>322.6</v>
       </c>
       <c r="E110" s="18" t="n">
@@ -5314,7 +5331,7 @@
       <c r="C111" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D111" s="17" t="n">
+      <c r="D111" s="49" t="n">
         <v>251.19</v>
       </c>
       <c r="E111" s="18" t="n">
@@ -5354,7 +5371,7 @@
       <c r="C112" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D112" s="17" t="n">
+      <c r="D112" s="49" t="n">
         <v>329.82</v>
       </c>
       <c r="E112" s="18" t="n">
@@ -5394,7 +5411,7 @@
       <c r="C113" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D113" s="17" t="n">
+      <c r="D113" s="49" t="n">
         <v>270.59</v>
       </c>
       <c r="E113" s="18" t="n">
@@ -5434,7 +5451,7 @@
       <c r="C114" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D114" s="17" t="n">
+      <c r="D114" s="49" t="n">
         <v>320.02</v>
       </c>
       <c r="E114" s="18" t="n">
@@ -5474,7 +5491,7 @@
       <c r="C115" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D115" s="17" t="n">
+      <c r="D115" s="49" t="n">
         <v>321.72</v>
       </c>
       <c r="E115" s="18" t="n">
@@ -5514,7 +5531,7 @@
       <c r="C116" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D116" s="17" t="n">
+      <c r="D116" s="49" t="n">
         <v>191.9</v>
       </c>
       <c r="E116" s="18" t="n">
@@ -5554,7 +5571,7 @@
       <c r="C117" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D117" s="17" t="n">
+      <c r="D117" s="49" t="n">
         <v>233.44</v>
       </c>
       <c r="E117" s="18" t="n">
@@ -5594,7 +5611,7 @@
       <c r="C118" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D118" s="17" t="n">
+      <c r="D118" s="49" t="n">
         <v>533.21</v>
       </c>
       <c r="E118" s="18" t="n">
@@ -5634,7 +5651,7 @@
       <c r="C119" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D119" s="17" t="n">
+      <c r="D119" s="49" t="n">
         <v>292.93</v>
       </c>
       <c r="E119" s="18" t="n">
@@ -5674,7 +5691,7 @@
       <c r="C120" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D120" s="17" t="n">
+      <c r="D120" s="49" t="n">
         <v>108.54</v>
       </c>
       <c r="E120" s="18" t="n">
@@ -5714,7 +5731,7 @@
       <c r="C121" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D121" s="17" t="n">
+      <c r="D121" s="49" t="n">
         <v>319.23</v>
       </c>
       <c r="E121" s="18" t="n">
@@ -5754,7 +5771,7 @@
       <c r="C122" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D122" s="17" t="n">
+      <c r="D122" s="49" t="n">
         <v>222.33</v>
       </c>
       <c r="E122" s="18" t="n">
@@ -5794,7 +5811,7 @@
       <c r="C123" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D123" s="17" t="n">
+      <c r="D123" s="49" t="n">
         <v>228.99</v>
       </c>
       <c r="E123" s="18" t="n">
@@ -5834,7 +5851,7 @@
       <c r="C124" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D124" s="17" t="n">
+      <c r="D124" s="49" t="n">
         <v>107.53</v>
       </c>
       <c r="E124" s="18" t="n">
@@ -5874,7 +5891,7 @@
       <c r="C125" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D125" s="17" t="n">
+      <c r="D125" s="49" t="n">
         <v>107.85</v>
       </c>
       <c r="E125" s="18" t="n">
@@ -5914,7 +5931,7 @@
       <c r="C126" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D126" s="17" t="n">
+      <c r="D126" s="49" t="n">
         <v>4.13</v>
       </c>
       <c r="E126" s="18" t="n">
@@ -5954,7 +5971,7 @@
       <c r="C127" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D127" s="17" t="n">
+      <c r="D127" s="49" t="n">
         <v>118.11</v>
       </c>
       <c r="E127" s="18" t="n">
@@ -5994,7 +6011,7 @@
       <c r="C128" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D128" s="17" t="n">
+      <c r="D128" s="49" t="n">
         <v>2.34</v>
       </c>
       <c r="E128" s="18" t="n">
@@ -6034,7 +6051,7 @@
       <c r="C129" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D129" s="17" t="n">
+      <c r="D129" s="49" t="n">
         <v>12.54</v>
       </c>
       <c r="E129" s="18" t="n">
@@ -6074,7 +6091,7 @@
       <c r="C130" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D130" s="17" t="n">
+      <c r="D130" s="49" t="n">
         <v>218.58</v>
       </c>
       <c r="E130" s="18" t="n">
@@ -6114,7 +6131,7 @@
       <c r="C131" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D131" s="17" t="n">
+      <c r="D131" s="49" t="n">
         <v>1.66</v>
       </c>
       <c r="E131" s="18" t="n">
@@ -6155,7 +6172,7 @@
         <f>SUM(C102:C131)</f>
         <v/>
       </c>
-      <c r="D132" s="22">
+      <c r="D132" s="50">
         <f>SUM(D102:D131)</f>
         <v/>
       </c>
@@ -6202,7 +6219,7 @@
       <c r="C133" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D133" s="17" t="n">
+      <c r="D133" s="49" t="n">
         <v>541.64</v>
       </c>
       <c r="E133" s="18" t="n">
@@ -6242,7 +6259,7 @@
       <c r="C134" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D134" s="17" t="n">
+      <c r="D134" s="49" t="n">
         <v>543.86</v>
       </c>
       <c r="E134" s="18" t="n">
@@ -6282,7 +6299,7 @@
       <c r="C135" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D135" s="17" t="n">
+      <c r="D135" s="49" t="n">
         <v>541.65</v>
       </c>
       <c r="E135" s="18" t="n">
@@ -6322,7 +6339,7 @@
       <c r="C136" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D136" s="17" t="n">
+      <c r="D136" s="49" t="n">
         <v>543.65</v>
       </c>
       <c r="E136" s="18" t="n">
@@ -6362,7 +6379,7 @@
       <c r="C137" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D137" s="17" t="n">
+      <c r="D137" s="49" t="n">
         <v>251.8</v>
       </c>
       <c r="E137" s="18" t="n">
@@ -6402,7 +6419,7 @@
       <c r="C138" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D138" s="17" t="n">
+      <c r="D138" s="49" t="n">
         <v>413.79</v>
       </c>
       <c r="E138" s="18" t="n">
@@ -6442,7 +6459,7 @@
       <c r="C139" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D139" s="17" t="n">
+      <c r="D139" s="49" t="n">
         <v>329.83</v>
       </c>
       <c r="E139" s="18" t="n">
@@ -6482,7 +6499,7 @@
       <c r="C140" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D140" s="17" t="n">
+      <c r="D140" s="49" t="n">
         <v>322.61</v>
       </c>
       <c r="E140" s="18" t="n">
@@ -6522,7 +6539,7 @@
       <c r="C141" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D141" s="17" t="n">
+      <c r="D141" s="49" t="n">
         <v>349.64</v>
       </c>
       <c r="E141" s="18" t="n">
@@ -6562,7 +6579,7 @@
       <c r="C142" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D142" s="17" t="n">
+      <c r="D142" s="49" t="n">
         <v>321.5</v>
       </c>
       <c r="E142" s="18" t="n">
@@ -6602,7 +6619,7 @@
       <c r="C143" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D143" s="17" t="n">
+      <c r="D143" s="49" t="n">
         <v>470.59</v>
       </c>
       <c r="E143" s="18" t="n">
@@ -6642,7 +6659,7 @@
       <c r="C144" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D144" s="17" t="n">
+      <c r="D144" s="49" t="n">
         <v>250.82</v>
       </c>
       <c r="E144" s="18" t="n">
@@ -6682,7 +6699,7 @@
       <c r="C145" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D145" s="17" t="n">
+      <c r="D145" s="49" t="n">
         <v>470.6</v>
       </c>
       <c r="E145" s="18" t="n">
@@ -6722,7 +6739,7 @@
       <c r="C146" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D146" s="17" t="n">
+      <c r="D146" s="49" t="n">
         <v>329.84</v>
       </c>
       <c r="E146" s="18" t="n">
@@ -6762,7 +6779,7 @@
       <c r="C147" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D147" s="17" t="n">
+      <c r="D147" s="49" t="n">
         <v>322.16</v>
       </c>
       <c r="E147" s="18" t="n">
@@ -6802,7 +6819,7 @@
       <c r="C148" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D148" s="17" t="n">
+      <c r="D148" s="49" t="n">
         <v>318.65</v>
       </c>
       <c r="E148" s="18" t="n">
@@ -6842,7 +6859,7 @@
       <c r="C149" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D149" s="17" t="n">
+      <c r="D149" s="49" t="n">
         <v>367.9</v>
       </c>
       <c r="E149" s="18" t="n">
@@ -6882,7 +6899,7 @@
       <c r="C150" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D150" s="17" t="n">
+      <c r="D150" s="49" t="n">
         <v>319.67</v>
       </c>
       <c r="E150" s="18" t="n">
@@ -6922,7 +6939,7 @@
       <c r="C151" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D151" s="17" t="n">
+      <c r="D151" s="49" t="n">
         <v>329.84</v>
       </c>
       <c r="E151" s="18" t="n">
@@ -6962,7 +6979,7 @@
       <c r="C152" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D152" s="17" t="n">
+      <c r="D152" s="49" t="n">
         <v>329.81</v>
       </c>
       <c r="E152" s="18" t="n">
@@ -7002,7 +7019,7 @@
       <c r="C153" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D153" s="17" t="n">
+      <c r="D153" s="49" t="n">
         <v>278.38</v>
       </c>
       <c r="E153" s="18" t="n">
@@ -7042,7 +7059,7 @@
       <c r="C154" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D154" s="17" t="n">
+      <c r="D154" s="49" t="n">
         <v>108.54</v>
       </c>
       <c r="E154" s="18" t="n">
@@ -7082,7 +7099,7 @@
       <c r="C155" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D155" s="17" t="n">
+      <c r="D155" s="49" t="n">
         <v>318.81</v>
       </c>
       <c r="E155" s="18" t="n">
@@ -7122,7 +7139,7 @@
       <c r="C156" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D156" s="17" t="n">
+      <c r="D156" s="49" t="n">
         <v>319.3</v>
       </c>
       <c r="E156" s="18" t="n">
@@ -7162,7 +7179,7 @@
       <c r="C157" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D157" s="17" t="n">
+      <c r="D157" s="49" t="n">
         <v>108.53</v>
       </c>
       <c r="E157" s="18" t="n">
@@ -7202,7 +7219,7 @@
       <c r="C158" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D158" s="17" t="n">
+      <c r="D158" s="49" t="n">
         <v>161.93</v>
       </c>
       <c r="E158" s="18" t="n">
@@ -7242,7 +7259,7 @@
       <c r="C159" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D159" s="17" t="n">
+      <c r="D159" s="49" t="n">
         <v>322.41</v>
       </c>
       <c r="E159" s="18" t="n">
@@ -7282,7 +7299,7 @@
       <c r="C160" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D160" s="17" t="n">
+      <c r="D160" s="49" t="n">
         <v>255.56</v>
       </c>
       <c r="E160" s="18" t="n">
@@ -7322,7 +7339,7 @@
       <c r="C161" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D161" s="17" t="n">
+      <c r="D161" s="49" t="n">
         <v>71.58</v>
       </c>
       <c r="E161" s="18" t="n">
@@ -7362,7 +7379,7 @@
       <c r="C162" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D162" s="17" t="n">
+      <c r="D162" s="49" t="n">
         <v>107.59</v>
       </c>
       <c r="E162" s="18" t="n">
@@ -7402,7 +7419,7 @@
       <c r="C163" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D163" s="17" t="n">
+      <c r="D163" s="49" t="n">
         <v>220.94</v>
       </c>
       <c r="E163" s="18" t="n">
@@ -7442,7 +7459,7 @@
       <c r="C164" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D164" s="17" t="n">
+      <c r="D164" s="49" t="n">
         <v>3.08</v>
       </c>
       <c r="E164" s="18" t="n">
@@ -7482,7 +7499,7 @@
       <c r="C165" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D165" s="17" t="n">
+      <c r="D165" s="49" t="n">
         <v>17.36</v>
       </c>
       <c r="E165" s="18" t="n">
@@ -7522,7 +7539,7 @@
       <c r="C166" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D166" s="17" t="n">
+      <c r="D166" s="49" t="n">
         <v>35.41</v>
       </c>
       <c r="E166" s="18" t="n">
@@ -7562,7 +7579,7 @@
       <c r="C167" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D167" s="17" t="n">
+      <c r="D167" s="49" t="n">
         <v>12.48</v>
       </c>
       <c r="E167" s="18" t="n">
@@ -7602,7 +7619,7 @@
       <c r="C168" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D168" s="17" t="n">
+      <c r="D168" s="49" t="n">
         <v>29.8</v>
       </c>
       <c r="E168" s="18" t="n">
@@ -7642,7 +7659,7 @@
       <c r="C169" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D169" s="17" t="n">
+      <c r="D169" s="49" t="n">
         <v>2.8</v>
       </c>
       <c r="E169" s="18" t="n">
@@ -7682,7 +7699,7 @@
       <c r="C170" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D170" s="17" t="n">
+      <c r="D170" s="49" t="n">
         <v>177.34</v>
       </c>
       <c r="E170" s="18" t="n">
@@ -7723,7 +7740,7 @@
         <f>SUM(C133:C170)</f>
         <v/>
       </c>
-      <c r="D171" s="22">
+      <c r="D171" s="50">
         <f>SUM(D133:D170)</f>
         <v/>
       </c>
@@ -7770,7 +7787,7 @@
       <c r="C172" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D172" s="17" t="n">
+      <c r="D172" s="49" t="n">
         <v>543.64</v>
       </c>
       <c r="E172" s="18" t="n">
@@ -7810,7 +7827,7 @@
       <c r="C173" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D173" s="17" t="n">
+      <c r="D173" s="49" t="n">
         <v>543.86</v>
       </c>
       <c r="E173" s="18" t="n">
@@ -7850,7 +7867,7 @@
       <c r="C174" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D174" s="17" t="n">
+      <c r="D174" s="49" t="n">
         <v>543.88</v>
       </c>
       <c r="E174" s="18" t="n">
@@ -7890,7 +7907,7 @@
       <c r="C175" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D175" s="17" t="n">
+      <c r="D175" s="49" t="n">
         <v>543.8</v>
       </c>
       <c r="E175" s="18" t="n">
@@ -7930,7 +7947,7 @@
       <c r="C176" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D176" s="17" t="n">
+      <c r="D176" s="49" t="n">
         <v>543.89</v>
       </c>
       <c r="E176" s="18" t="n">
@@ -7970,7 +7987,7 @@
       <c r="C177" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D177" s="17" t="n">
+      <c r="D177" s="49" t="n">
         <v>543.88</v>
       </c>
       <c r="E177" s="18" t="n">
@@ -8010,7 +8027,7 @@
       <c r="C178" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D178" s="17" t="n">
+      <c r="D178" s="49" t="n">
         <v>543.89</v>
       </c>
       <c r="E178" s="18" t="n">
@@ -8050,7 +8067,7 @@
       <c r="C179" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D179" s="17" t="n">
+      <c r="D179" s="49" t="n">
         <v>251.79</v>
       </c>
       <c r="E179" s="18" t="n">
@@ -8090,7 +8107,7 @@
       <c r="C180" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D180" s="17" t="n">
+      <c r="D180" s="49" t="n">
         <v>251.91</v>
       </c>
       <c r="E180" s="18" t="n">
@@ -8130,7 +8147,7 @@
       <c r="C181" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D181" s="17" t="n">
+      <c r="D181" s="49" t="n">
         <v>329.84</v>
       </c>
       <c r="E181" s="18" t="n">
@@ -8170,7 +8187,7 @@
       <c r="C182" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D182" s="17" t="n">
+      <c r="D182" s="49" t="n">
         <v>322.6</v>
       </c>
       <c r="E182" s="18" t="n">
@@ -8210,7 +8227,7 @@
       <c r="C183" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D183" s="17" t="n">
+      <c r="D183" s="49" t="n">
         <v>469.9</v>
       </c>
       <c r="E183" s="18" t="n">
@@ -8250,7 +8267,7 @@
       <c r="C184" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D184" s="17" t="n">
+      <c r="D184" s="49" t="n">
         <v>321.48</v>
       </c>
       <c r="E184" s="18" t="n">
@@ -8290,7 +8307,7 @@
       <c r="C185" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D185" s="17" t="n">
+      <c r="D185" s="49" t="n">
         <v>473.49</v>
       </c>
       <c r="E185" s="18" t="n">
@@ -8330,7 +8347,7 @@
       <c r="C186" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D186" s="17" t="n">
+      <c r="D186" s="49" t="n">
         <v>329.79</v>
       </c>
       <c r="E186" s="18" t="n">
@@ -8370,7 +8387,7 @@
       <c r="C187" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D187" s="17" t="n">
+      <c r="D187" s="49" t="n">
         <v>470.58</v>
       </c>
       <c r="E187" s="18" t="n">
@@ -8410,7 +8427,7 @@
       <c r="C188" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D188" s="17" t="n">
+      <c r="D188" s="49" t="n">
         <v>221.64</v>
       </c>
       <c r="E188" s="18" t="n">
@@ -8450,7 +8467,7 @@
       <c r="C189" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D189" s="17" t="n">
+      <c r="D189" s="49" t="n">
         <v>319.18</v>
       </c>
       <c r="E189" s="18" t="n">
@@ -8490,7 +8507,7 @@
       <c r="C190" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D190" s="17" t="n">
+      <c r="D190" s="49" t="n">
         <v>320.03</v>
       </c>
       <c r="E190" s="18" t="n">
@@ -8530,7 +8547,7 @@
       <c r="C191" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D191" s="17" t="n">
+      <c r="D191" s="49" t="n">
         <v>321.7</v>
       </c>
       <c r="E191" s="18" t="n">
@@ -8570,7 +8587,7 @@
       <c r="C192" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D192" s="17" t="n">
+      <c r="D192" s="49" t="n">
         <v>194.26</v>
       </c>
       <c r="E192" s="18" t="n">
@@ -8610,7 +8627,7 @@
       <c r="C193" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D193" s="17" t="n">
+      <c r="D193" s="49" t="n">
         <v>108.54</v>
       </c>
       <c r="E193" s="18" t="n">
@@ -8650,7 +8667,7 @@
       <c r="C194" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D194" s="17" t="n">
+      <c r="D194" s="49" t="n">
         <v>108.58</v>
       </c>
       <c r="E194" s="18" t="n">
@@ -8690,7 +8707,7 @@
       <c r="C195" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D195" s="17" t="n">
+      <c r="D195" s="49" t="n">
         <v>156.1</v>
       </c>
       <c r="E195" s="18" t="n">
@@ -8730,7 +8747,7 @@
       <c r="C196" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D196" s="17" t="n">
+      <c r="D196" s="49" t="n">
         <v>205.92</v>
       </c>
       <c r="E196" s="18" t="n">
@@ -8770,7 +8787,7 @@
       <c r="C197" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D197" s="17" t="n">
+      <c r="D197" s="49" t="n">
         <v>222.25</v>
       </c>
       <c r="E197" s="18" t="n">
@@ -8810,7 +8827,7 @@
       <c r="C198" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D198" s="17" t="n">
+      <c r="D198" s="49" t="n">
         <v>167.18</v>
       </c>
       <c r="E198" s="18" t="n">
@@ -8850,7 +8867,7 @@
       <c r="C199" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D199" s="17" t="n">
+      <c r="D199" s="49" t="n">
         <v>127.68</v>
       </c>
       <c r="E199" s="18" t="n">
@@ -8890,7 +8907,7 @@
       <c r="C200" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D200" s="17" t="n">
+      <c r="D200" s="49" t="n">
         <v>77.84999999999999</v>
       </c>
       <c r="E200" s="18" t="n">
@@ -8930,7 +8947,7 @@
       <c r="C201" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D201" s="17" t="n">
+      <c r="D201" s="49" t="n">
         <v>47.08</v>
       </c>
       <c r="E201" s="18" t="n">
@@ -8970,7 +8987,7 @@
       <c r="C202" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D202" s="17" t="n">
+      <c r="D202" s="49" t="n">
         <v>101.41</v>
       </c>
       <c r="E202" s="18" t="n">
@@ -9010,7 +9027,7 @@
       <c r="C203" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D203" s="17" t="n">
+      <c r="D203" s="49" t="n">
         <v>32.79</v>
       </c>
       <c r="E203" s="18" t="n">
@@ -9050,7 +9067,7 @@
       <c r="C204" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D204" s="17" t="n">
+      <c r="D204" s="49" t="n">
         <v>67.19</v>
       </c>
       <c r="E204" s="18" t="n">
@@ -9090,7 +9107,7 @@
       <c r="C205" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D205" s="17" t="n">
+      <c r="D205" s="49" t="n">
         <v>52.23</v>
       </c>
       <c r="E205" s="18" t="n">
@@ -9130,7 +9147,7 @@
       <c r="C206" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D206" s="17" t="n">
+      <c r="D206" s="49" t="n">
         <v>12.15</v>
       </c>
       <c r="E206" s="18" t="n">
@@ -9170,7 +9187,7 @@
       <c r="C207" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D207" s="17" t="n">
+      <c r="D207" s="49" t="n">
         <v>25.67</v>
       </c>
       <c r="E207" s="18" t="n">
@@ -9210,7 +9227,7 @@
       <c r="C208" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D208" s="17" t="n">
+      <c r="D208" s="49" t="n">
         <v>72.69</v>
       </c>
       <c r="E208" s="18" t="n">
@@ -9250,7 +9267,7 @@
       <c r="C209" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D209" s="17" t="n">
+      <c r="D209" s="49" t="n">
         <v>62.47</v>
       </c>
       <c r="E209" s="18" t="n">
@@ -9290,7 +9307,7 @@
       <c r="C210" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D210" s="17" t="n">
+      <c r="D210" s="49" t="n">
         <v>139.49</v>
       </c>
       <c r="E210" s="18" t="n">
@@ -9330,7 +9347,7 @@
       <c r="C211" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D211" s="17" t="n">
+      <c r="D211" s="49" t="n">
         <v>28.86</v>
       </c>
       <c r="E211" s="18" t="n">
@@ -9371,7 +9388,7 @@
         <f>SUM(C172:C211)</f>
         <v/>
       </c>
-      <c r="D212" s="22">
+      <c r="D212" s="50">
         <f>SUM(D172:D211)</f>
         <v/>
       </c>
@@ -9418,7 +9435,7 @@
       <c r="C213" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D213" s="17" t="n">
+      <c r="D213" s="49" t="n">
         <v>543.86</v>
       </c>
       <c r="E213" s="18" t="n">
@@ -9458,7 +9475,7 @@
       <c r="C214" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D214" s="17" t="n">
+      <c r="D214" s="49" t="n">
         <v>541.65</v>
       </c>
       <c r="E214" s="18" t="n">
@@ -9498,7 +9515,7 @@
       <c r="C215" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D215" s="17" t="n">
+      <c r="D215" s="49" t="n">
         <v>543.88</v>
       </c>
       <c r="E215" s="18" t="n">
@@ -9538,7 +9555,7 @@
       <c r="C216" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D216" s="17" t="n">
+      <c r="D216" s="49" t="n">
         <v>541.65</v>
       </c>
       <c r="E216" s="18" t="n">
@@ -9578,7 +9595,7 @@
       <c r="C217" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D217" s="17" t="n">
+      <c r="D217" s="49" t="n">
         <v>543.65</v>
       </c>
       <c r="E217" s="18" t="n">
@@ -9618,7 +9635,7 @@
       <c r="C218" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D218" s="17" t="n">
+      <c r="D218" s="49" t="n">
         <v>543.89</v>
       </c>
       <c r="E218" s="18" t="n">
@@ -9658,7 +9675,7 @@
       <c r="C219" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D219" s="17" t="n">
+      <c r="D219" s="49" t="n">
         <v>251.32</v>
       </c>
       <c r="E219" s="18" t="n">
@@ -9698,7 +9715,7 @@
       <c r="C220" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D220" s="17" t="n">
+      <c r="D220" s="49" t="n">
         <v>252.05</v>
       </c>
       <c r="E220" s="18" t="n">
@@ -9738,7 +9755,7 @@
       <c r="C221" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D221" s="17" t="n">
+      <c r="D221" s="49" t="n">
         <v>515.48</v>
       </c>
       <c r="E221" s="18" t="n">
@@ -9778,7 +9795,7 @@
       <c r="C222" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D222" s="17" t="n">
+      <c r="D222" s="49" t="n">
         <v>329.84</v>
       </c>
       <c r="E222" s="18" t="n">
@@ -9818,7 +9835,7 @@
       <c r="C223" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D223" s="17" t="n">
+      <c r="D223" s="49" t="n">
         <v>184.4</v>
       </c>
       <c r="E223" s="18" t="n">
@@ -9858,7 +9875,7 @@
       <c r="C224" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D224" s="17" t="n">
+      <c r="D224" s="49" t="n">
         <v>321.5</v>
       </c>
       <c r="E224" s="18" t="n">
@@ -9898,7 +9915,7 @@
       <c r="C225" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D225" s="17" t="n">
+      <c r="D225" s="49" t="n">
         <v>387.98</v>
       </c>
       <c r="E225" s="18" t="n">
@@ -9938,7 +9955,7 @@
       <c r="C226" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D226" s="17" t="n">
+      <c r="D226" s="49" t="n">
         <v>330.17</v>
       </c>
       <c r="E226" s="18" t="n">
@@ -9978,7 +9995,7 @@
       <c r="C227" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D227" s="17" t="n">
+      <c r="D227" s="49" t="n">
         <v>513</v>
       </c>
       <c r="E227" s="18" t="n">
@@ -10018,7 +10035,7 @@
       <c r="C228" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D228" s="17" t="n">
+      <c r="D228" s="49" t="n">
         <v>473.44</v>
       </c>
       <c r="E228" s="18" t="n">
@@ -10058,7 +10075,7 @@
       <c r="C229" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D229" s="17" t="n">
+      <c r="D229" s="49" t="n">
         <v>463.93</v>
       </c>
       <c r="E229" s="18" t="n">
@@ -10098,7 +10115,7 @@
       <c r="C230" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D230" s="17" t="n">
+      <c r="D230" s="49" t="n">
         <v>486.72</v>
       </c>
       <c r="E230" s="18" t="n">
@@ -10138,7 +10155,7 @@
       <c r="C231" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D231" s="17" t="n">
+      <c r="D231" s="49" t="n">
         <v>470.58</v>
       </c>
       <c r="E231" s="18" t="n">
@@ -10178,7 +10195,7 @@
       <c r="C232" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D232" s="17" t="n">
+      <c r="D232" s="49" t="n">
         <v>454.84</v>
       </c>
       <c r="E232" s="18" t="n">
@@ -10218,7 +10235,7 @@
       <c r="C233" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D233" s="17" t="n">
+      <c r="D233" s="49" t="n">
         <v>476.45</v>
       </c>
       <c r="E233" s="18" t="n">
@@ -10258,7 +10275,7 @@
       <c r="C234" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D234" s="17" t="n">
+      <c r="D234" s="49" t="n">
         <v>219.34</v>
       </c>
       <c r="E234" s="18" t="n">
@@ -10298,7 +10315,7 @@
       <c r="C235" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D235" s="17" t="n">
+      <c r="D235" s="49" t="n">
         <v>348.76</v>
       </c>
       <c r="E235" s="18" t="n">
@@ -10338,7 +10355,7 @@
       <c r="C236" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D236" s="17" t="n">
+      <c r="D236" s="49" t="n">
         <v>318.81</v>
       </c>
       <c r="E236" s="18" t="n">
@@ -10378,7 +10395,7 @@
       <c r="C237" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D237" s="17" t="n">
+      <c r="D237" s="49" t="n">
         <v>264.61</v>
       </c>
       <c r="E237" s="18" t="n">
@@ -10418,7 +10435,7 @@
       <c r="C238" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D238" s="17" t="n">
+      <c r="D238" s="49" t="n">
         <v>108.67</v>
       </c>
       <c r="E238" s="18" t="n">
@@ -10458,7 +10475,7 @@
       <c r="C239" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D239" s="17" t="n">
+      <c r="D239" s="49" t="n">
         <v>229.72</v>
       </c>
       <c r="E239" s="18" t="n">
@@ -10498,7 +10515,7 @@
       <c r="C240" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D240" s="17" t="n">
+      <c r="D240" s="49" t="n">
         <v>304.18</v>
       </c>
       <c r="E240" s="18" t="n">
@@ -10538,7 +10555,7 @@
       <c r="C241" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D241" s="17" t="n">
+      <c r="D241" s="49" t="n">
         <v>322.63</v>
       </c>
       <c r="E241" s="18" t="n">
@@ -10578,7 +10595,7 @@
       <c r="C242" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D242" s="17" t="n">
+      <c r="D242" s="49" t="n">
         <v>313.1</v>
       </c>
       <c r="E242" s="18" t="n">
@@ -10618,7 +10635,7 @@
       <c r="C243" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D243" s="17" t="n">
+      <c r="D243" s="49" t="n">
         <v>201.72</v>
       </c>
       <c r="E243" s="18" t="n">
@@ -10658,7 +10675,7 @@
       <c r="C244" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D244" s="17" t="n">
+      <c r="D244" s="49" t="n">
         <v>108.52</v>
       </c>
       <c r="E244" s="18" t="n">
@@ -10698,7 +10715,7 @@
       <c r="C245" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D245" s="17" t="n">
+      <c r="D245" s="49" t="n">
         <v>88.45999999999999</v>
       </c>
       <c r="E245" s="18" t="n">
@@ -10738,7 +10755,7 @@
       <c r="C246" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D246" s="17" t="n">
+      <c r="D246" s="49" t="n">
         <v>189.22</v>
       </c>
       <c r="E246" s="18" t="n">
@@ -10778,7 +10795,7 @@
       <c r="C247" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D247" s="17" t="n">
+      <c r="D247" s="49" t="n">
         <v>40.28</v>
       </c>
       <c r="E247" s="18" t="n">
@@ -10818,7 +10835,7 @@
       <c r="C248" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D248" s="17" t="n">
+      <c r="D248" s="49" t="n">
         <v>77.34999999999999</v>
       </c>
       <c r="E248" s="18" t="n">
@@ -10858,7 +10875,7 @@
       <c r="C249" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D249" s="17" t="n">
+      <c r="D249" s="49" t="n">
         <v>36.32</v>
       </c>
       <c r="E249" s="18" t="n">
@@ -10898,7 +10915,7 @@
       <c r="C250" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D250" s="17" t="n">
+      <c r="D250" s="49" t="n">
         <v>32.74</v>
       </c>
       <c r="E250" s="18" t="n">
@@ -10938,7 +10955,7 @@
       <c r="C251" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D251" s="17" t="n">
+      <c r="D251" s="49" t="n">
         <v>0.22</v>
       </c>
       <c r="E251" s="18" t="n">
@@ -10979,7 +10996,7 @@
         <f>SUM(C213:C251)</f>
         <v/>
       </c>
-      <c r="D252" s="22">
+      <c r="D252" s="50">
         <f>SUM(D213:D251)</f>
         <v/>
       </c>
@@ -11023,7 +11040,7 @@
         <f>C39+C69+C101+C132+C171+C212+C252</f>
         <v/>
       </c>
-      <c r="D253" s="27">
+      <c r="D253" s="51">
         <f>D39+D69+D101+D132+D171+D212+D252</f>
         <v/>
       </c>
@@ -11105,7 +11122,7 @@
     <row r="3">
       <c r="A3" s="30" t="inlineStr">
         <is>
-          <t>Total EB = 34   ·   Valid trips = 5   ·   Non-valid trips = 29   ·   Undesirable = 26</t>
+          <t>Total EB = 34   ·   Valid trips = 5   ·   Non-valid trips = 29   ·   Undesirable = 29</t>
         </is>
       </c>
     </row>
@@ -11644,7 +11661,7 @@
       </c>
       <c r="P10" s="33" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>StandBy Mode</t>
         </is>
       </c>
       <c r="Q10" s="33" t="inlineStr">
@@ -11735,7 +11752,7 @@
       </c>
       <c r="P11" s="33" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>StandBy Mode</t>
         </is>
       </c>
       <c r="Q11" s="33" t="inlineStr">
@@ -14289,7 +14306,7 @@
       </c>
       <c r="P39" s="33" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>StandBy Mode</t>
         </is>
       </c>
       <c r="Q39" s="33" t="inlineStr">
@@ -14357,7 +14374,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -34787,7 +34803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="B1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -34802,7 +34818,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="34" customHeight="1">
       <c r="B3" s="44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
update WCR dashboard data 2026-07-01 11:48
</commit_message>
<xml_diff>
--- a/docs/reports/WCR_Kavach_Unified_KPI_Jun1-Jun7.xlsx
+++ b/docs/reports/WCR_Kavach_Unified_KPI_Jun1-Jun7.xlsx
@@ -731,7 +731,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -956,6 +955,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="37" t="inlineStr">
+        <is>
+          <t>Availability base excludes locos with FS+OS pkts = 0 (they are still listed; only the Total-pkts availability base drops them).</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -2437,7 +2443,7 @@
         <v/>
       </c>
       <c r="F39" s="23">
-        <f>SUM(F4:F38)</f>
+        <f>SUMIF(E4:E38,"&gt;0",F4:F38)</f>
         <v/>
       </c>
       <c r="G39" s="24">
@@ -3645,7 +3651,7 @@
         <v/>
       </c>
       <c r="F69" s="23">
-        <f>SUM(F40:F68)</f>
+        <f>SUMIF(E40:E68,"&gt;0",F40:F68)</f>
         <v/>
       </c>
       <c r="G69" s="24">
@@ -4933,7 +4939,7 @@
         <v/>
       </c>
       <c r="F101" s="23">
-        <f>SUM(F70:F100)</f>
+        <f>SUMIF(E70:E100,"&gt;0",F70:F100)</f>
         <v/>
       </c>
       <c r="G101" s="24">
@@ -6181,7 +6187,7 @@
         <v/>
       </c>
       <c r="F132" s="23">
-        <f>SUM(F102:F131)</f>
+        <f>SUMIF(E102:E131,"&gt;0",F102:F131)</f>
         <v/>
       </c>
       <c r="G132" s="24">
@@ -7749,7 +7755,7 @@
         <v/>
       </c>
       <c r="F171" s="23">
-        <f>SUM(F133:F170)</f>
+        <f>SUMIF(E133:E170,"&gt;0",F133:F170)</f>
         <v/>
       </c>
       <c r="G171" s="24">
@@ -9397,7 +9403,7 @@
         <v/>
       </c>
       <c r="F212" s="23">
-        <f>SUM(F172:F211)</f>
+        <f>SUMIF(E172:E211,"&gt;0",F172:F211)</f>
         <v/>
       </c>
       <c r="G212" s="24">
@@ -11005,7 +11011,7 @@
         <v/>
       </c>
       <c r="F252" s="23">
-        <f>SUM(F213:F251)</f>
+        <f>SUMIF(E213:E251,"&gt;0",F213:F251)</f>
         <v/>
       </c>
       <c r="G252" s="24">
@@ -11118,7 +11124,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="30" t="inlineStr">
         <is>
@@ -11126,7 +11131,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>

</xml_diff>